<commit_message>
Update GCD Csp flattest-window analysis
</commit_message>
<xml_diff>
--- a/data/processed/GCD/tables/hBN_GCD_bounded_fit_summary_final.xlsx
+++ b/data/processed/GCD/tables/hBN_GCD_bounded_fit_summary_final.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,90 +444,100 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>window_selection_method</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>flatness_score</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>V0_base_V</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Rs_base_ohm</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>effective_IR_drop_base_mV</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Csp_base_F_g^-1</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>A_base</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>tau_base_s</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Csp_CI2.5_F_g^-1</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Csp_median_F_g^-1</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Csp_CI97.5_F_g^-1</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>IRdrop_CI2.5_mV</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>IRdrop_median_mV</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>IRdrop_CI97.5_mV</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>A_CI2.5</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>A_median</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>A_CI97.5</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>tau_CI2.5_s</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>tau_median_s</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>tau_CI97.5_s</t>
         </is>
@@ -538,69 +548,77 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1.020404070033699</v>
+        <v>2.480403420049704</v>
       </c>
       <c r="C2" t="n">
-        <v>10.1904039400397</v>
+        <v>9.660403930000101</v>
       </c>
       <c r="D2" t="n">
-        <v>9.169999870006</v>
+        <v>7.180000509950396</v>
       </c>
       <c r="E2" t="n">
-        <v>918</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.2808998495376823</v>
+        <v>719</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>flattest_linear_post_ir_window</t>
+        </is>
       </c>
       <c r="G2" t="n">
+        <v>0.4090083896037332</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.2537316398228566</v>
+      </c>
+      <c r="I2" t="n">
         <v>0.009867003129131019</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>9.867003129131019</v>
       </c>
-      <c r="I2" t="n">
-        <v>82.08268396494205</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
       <c r="K2" t="n">
-        <v>9</v>
+        <v>99.0876457235766</v>
       </c>
       <c r="L2" t="n">
-        <v>80.31299522823559</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>82.11277905247866</v>
+        <v>9</v>
       </c>
       <c r="N2" t="n">
-        <v>84.47052639463416</v>
+        <v>98.6000265889823</v>
       </c>
       <c r="O2" t="n">
-        <v>9.867003129131019</v>
+        <v>99.1286302705513</v>
       </c>
       <c r="P2" t="n">
-        <v>9.867003129131019</v>
+        <v>99.65238835783501</v>
       </c>
       <c r="Q2" t="n">
         <v>9.867003129131019</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>9.867003129131019</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>9.867003129131019</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W2" t="n">
+        <v>9</v>
+      </c>
+      <c r="X2" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -609,69 +627,77 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.6164643500233069</v>
+        <v>1.294464180013208</v>
       </c>
       <c r="C3" t="n">
-        <v>5.126464340020903</v>
+        <v>4.601464139996096</v>
       </c>
       <c r="D3" t="n">
-        <v>4.509999989997596</v>
+        <v>3.306999959982889</v>
       </c>
       <c r="E3" t="n">
-        <v>4511</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.2837189520967451</v>
+        <v>3308</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>flattest_linear_post_ir_window</t>
+        </is>
       </c>
       <c r="G3" t="n">
+        <v>0.2976232637509973</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.2618697187305725</v>
+      </c>
+      <c r="I3" t="n">
         <v>0.009732716467688456</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>19.46543293537691</v>
       </c>
-      <c r="I3" t="n">
-        <v>80.75702396739435</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
       <c r="K3" t="n">
-        <v>9</v>
+        <v>90.02908328210498</v>
       </c>
       <c r="L3" t="n">
-        <v>80.20990188044964</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>80.74670051650878</v>
+        <v>9</v>
       </c>
       <c r="N3" t="n">
-        <v>81.19577048147131</v>
+        <v>89.9074379826454</v>
       </c>
       <c r="O3" t="n">
-        <v>19.46543293537691</v>
+        <v>90.01538059959415</v>
       </c>
       <c r="P3" t="n">
-        <v>19.46543293537691</v>
+        <v>90.13615425000829</v>
       </c>
       <c r="Q3" t="n">
         <v>19.46543293537691</v>
       </c>
       <c r="R3" t="n">
-        <v>0</v>
+        <v>19.46543293537691</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>19.46543293537691</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W3" t="n">
+        <v>9</v>
+      </c>
+      <c r="X3" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -680,69 +706,77 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4754521000440088</v>
+        <v>0.8774522900350088</v>
       </c>
       <c r="C4" t="n">
-        <v>3.388452050044009</v>
+        <v>2.880452080048002</v>
       </c>
       <c r="D4" t="n">
-        <v>2.91299995</v>
+        <v>2.002999790012993</v>
       </c>
       <c r="E4" t="n">
-        <v>2914</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.2888111214176615</v>
+        <v>2004</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>flattest_linear_post_ir_window</t>
+        </is>
       </c>
       <c r="G4" t="n">
+        <v>0.2681048894817717</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.2704394929563628</v>
+      </c>
+      <c r="I4" t="n">
         <v>0.009627444607500105</v>
       </c>
-      <c r="H4" t="n">
+      <c r="J4" t="n">
         <v>28.88233382250031</v>
       </c>
-      <c r="I4" t="n">
-        <v>76.6425806985272</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
       <c r="K4" t="n">
-        <v>9</v>
+        <v>82.62651540927513</v>
       </c>
       <c r="L4" t="n">
-        <v>76.17881501183567</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>76.63791828889543</v>
+        <v>9</v>
       </c>
       <c r="N4" t="n">
-        <v>77.05125729670256</v>
+        <v>82.5122170999024</v>
       </c>
       <c r="O4" t="n">
-        <v>28.88233382250031</v>
+        <v>82.61649094540422</v>
       </c>
       <c r="P4" t="n">
-        <v>28.88233382250031</v>
+        <v>82.72682779643704</v>
       </c>
       <c r="Q4" t="n">
         <v>28.88233382250031</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>28.88233382250031</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>28.88233382250031</v>
       </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W4" t="n">
+        <v>9</v>
+      </c>
+      <c r="X4" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y4" t="n">
         <v>9</v>
       </c>
     </row>
@@ -751,69 +785,77 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.410445009940986</v>
+        <v>1.111445009942003</v>
       </c>
       <c r="C5" t="n">
-        <v>2.507445010007985</v>
+        <v>2.225445410004</v>
       </c>
       <c r="D5" t="n">
-        <v>2.097000000066999</v>
+        <v>1.114000400061997</v>
       </c>
       <c r="E5" t="n">
-        <v>2098</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.2940145966772055</v>
+        <v>1115</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>flattest_linear_post_ir_window</t>
+        </is>
       </c>
       <c r="G5" t="n">
+        <v>0.2966933910250072</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.2578444668184073</v>
+      </c>
+      <c r="I5" t="n">
         <v>0.009465826381994863</v>
       </c>
-      <c r="H5" t="n">
+      <c r="J5" t="n">
         <v>37.86330552797945</v>
       </c>
-      <c r="I5" t="n">
-        <v>71.8581587139351</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
       <c r="K5" t="n">
-        <v>9</v>
+        <v>70.89006794626557</v>
       </c>
       <c r="L5" t="n">
-        <v>71.41374029367795</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>71.90173617620096</v>
+        <v>9</v>
       </c>
       <c r="N5" t="n">
-        <v>72.27242579298996</v>
+        <v>70.75556429483144</v>
       </c>
       <c r="O5" t="n">
-        <v>37.86330552797945</v>
+        <v>70.87888864609477</v>
       </c>
       <c r="P5" t="n">
-        <v>37.86330552797945</v>
+        <v>71.08057868838678</v>
       </c>
       <c r="Q5" t="n">
         <v>37.86330552797945</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>37.86330552797945</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>37.86330552797945</v>
       </c>
       <c r="T5" t="n">
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W5" t="n">
+        <v>9</v>
+      </c>
+      <c r="X5" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y5" t="n">
         <v>9</v>
       </c>
     </row>
@@ -822,69 +864,77 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>0.4004157399759833</v>
+        <v>1.011415569926982</v>
       </c>
       <c r="C6" t="n">
-        <v>1.974415799951998</v>
+        <v>1.741415560012996</v>
       </c>
       <c r="D6" t="n">
-        <v>1.574000059976015</v>
+        <v>0.7299999900860143</v>
       </c>
       <c r="E6" t="n">
-        <v>1575</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.2978504356018702</v>
+        <v>731</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>flattest_linear_post_ir_window</t>
+        </is>
       </c>
       <c r="G6" t="n">
+        <v>0.3329790938609002</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.2578480005956012</v>
+      </c>
+      <c r="I6" t="n">
         <v>0.009339393602113992</v>
       </c>
-      <c r="H6" t="n">
+      <c r="J6" t="n">
         <v>46.69696801056996</v>
       </c>
-      <c r="I6" t="n">
-        <v>66.63859685454328</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
       <c r="K6" t="n">
-        <v>9</v>
+        <v>61.27702420765139</v>
       </c>
       <c r="L6" t="n">
-        <v>65.89827369558307</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>66.62799103208224</v>
+        <v>9</v>
       </c>
       <c r="N6" t="n">
-        <v>67.15924219289856</v>
+        <v>60.92660592733132</v>
       </c>
       <c r="O6" t="n">
-        <v>46.69696801056996</v>
+        <v>61.23915218415829</v>
       </c>
       <c r="P6" t="n">
-        <v>46.69696801056996</v>
+        <v>61.53005294342042</v>
       </c>
       <c r="Q6" t="n">
         <v>46.69696801056996</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>46.69696801056996</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>46.69696801056996</v>
       </c>
       <c r="T6" t="n">
         <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W6" t="n">
+        <v>9</v>
+      </c>
+      <c r="X6" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y6" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Address PR 20 review comments
</commit_message>
<xml_diff>
--- a/data/processed/GCD/tables/hBN_GCD_bounded_fit_summary_final.xlsx
+++ b/data/processed/GCD/tables/hBN_GCD_bounded_fit_summary_final.xlsx
@@ -586,13 +586,13 @@
         <v>9</v>
       </c>
       <c r="N2" t="n">
-        <v>98.6000265889823</v>
+        <v>98.6000265889824</v>
       </c>
       <c r="O2" t="n">
-        <v>99.1286302705513</v>
+        <v>99.12863027055167</v>
       </c>
       <c r="P2" t="n">
-        <v>99.65238835783501</v>
+        <v>99.65238835783461</v>
       </c>
       <c r="Q2" t="n">
         <v>9.867003129131019</v>
@@ -665,13 +665,13 @@
         <v>9</v>
       </c>
       <c r="N3" t="n">
-        <v>89.9074379826454</v>
+        <v>89.90743798264548</v>
       </c>
       <c r="O3" t="n">
-        <v>90.01538059959415</v>
+        <v>90.01538059959385</v>
       </c>
       <c r="P3" t="n">
-        <v>90.13615425000829</v>
+        <v>90.13615425000822</v>
       </c>
       <c r="Q3" t="n">
         <v>19.46543293537691</v>
@@ -744,13 +744,13 @@
         <v>9</v>
       </c>
       <c r="N4" t="n">
-        <v>82.5122170999024</v>
+        <v>82.51221709990232</v>
       </c>
       <c r="O4" t="n">
-        <v>82.61649094540422</v>
+        <v>82.61649094540415</v>
       </c>
       <c r="P4" t="n">
-        <v>82.72682779643704</v>
+        <v>82.72682779643702</v>
       </c>
       <c r="Q4" t="n">
         <v>28.88233382250031</v>
@@ -823,13 +823,13 @@
         <v>9</v>
       </c>
       <c r="N5" t="n">
-        <v>70.75556429483144</v>
+        <v>70.75556429483119</v>
       </c>
       <c r="O5" t="n">
-        <v>70.87888864609477</v>
+        <v>70.87888864609494</v>
       </c>
       <c r="P5" t="n">
-        <v>71.08057868838678</v>
+        <v>71.08057868838701</v>
       </c>
       <c r="Q5" t="n">
         <v>37.86330552797945</v>
@@ -902,13 +902,13 @@
         <v>9</v>
       </c>
       <c r="N6" t="n">
-        <v>60.92660592733132</v>
+        <v>60.92660592733156</v>
       </c>
       <c r="O6" t="n">
-        <v>61.23915218415829</v>
+        <v>61.2391521841581</v>
       </c>
       <c r="P6" t="n">
-        <v>61.53005294342042</v>
+        <v>61.5300529434202</v>
       </c>
       <c r="Q6" t="n">
         <v>46.69696801056996</v>

</xml_diff>